<commit_message>
Correct XBB.1.5.77 in voc1 to XBB.1.5.72
</commit_message>
<xml_diff>
--- a/Lineage_Colors_on_CDT.xlsx
+++ b/Lineage_Colors_on_CDT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\repos\sc2_proportion_modeling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2EAF722-C5E3-4E78-8510-1FEF0C2435D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED6DA15-A2FF-42BD-9F69-6B5D4AA60341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14595" yWindow="705" windowWidth="16545" windowHeight="14340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15510" yWindow="2220" windowWidth="10785" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lineage Summary" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t>Variant</t>
   </si>
@@ -188,13 +188,61 @@
   </si>
   <si>
     <t>#827717</t>
+  </si>
+  <si>
+    <t>XBB.1.5.10</t>
+  </si>
+  <si>
+    <t>#f97a57</t>
+  </si>
+  <si>
+    <t>EU.1.1</t>
+  </si>
+  <si>
+    <t>#f25353</t>
+  </si>
+  <si>
+    <t>XBB.1.5.68</t>
+  </si>
+  <si>
+    <t>#86bcb6</t>
+  </si>
+  <si>
+    <t>FE.1.1</t>
+  </si>
+  <si>
+    <t>#499894</t>
+  </si>
+  <si>
+    <t>EG.5</t>
+  </si>
+  <si>
+    <t>#f28e2b</t>
+  </si>
+  <si>
+    <t>XBB.1.5.59</t>
+  </si>
+  <si>
+    <t>#ffbe7d</t>
+  </si>
+  <si>
+    <t>XBB.1.16.6</t>
+  </si>
+  <si>
+    <t>#59a14f</t>
+  </si>
+  <si>
+    <t>XBB.1.5.72</t>
+  </si>
+  <si>
+    <t>#254220</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -332,12 +380,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -698,12 +740,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1066,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -1082,219 +1121,283 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B24" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B25" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>41</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B26" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B27" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B28" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B30" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B31" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B32" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>66</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1521,15 +1624,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd">
@@ -1538,6 +1632,15 @@
     <TaxCatchAll xmlns="90bc503b-6eb4-4477-9236-230e894a8c79" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1560,14 +1663,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECE872C0-CA59-4E8E-8928-E8AC0DA3AB58}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D14E7338-C7ED-4988-977F-AB8C51D5B02E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1576,4 +1671,12 @@
     <ds:schemaRef ds:uri="90bc503b-6eb4-4477-9236-230e894a8c79"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECE872C0-CA59-4E8E-8928-E8AC0DA3AB58}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Production runs: 2023-08-08, The parent lineage colors has been updated
</commit_message>
<xml_diff>
--- a/Lineage_Colors_on_CDT.xlsx
+++ b/Lineage_Colors_on_CDT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\repos\sc2_proportion_modeling\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\groups.biotech.cdc.gov\groups\Projects\SARS2Seq\repos\sc2_proportion_modeling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED6DA15-A2FF-42BD-9F69-6B5D4AA60341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE603992-250F-4C6D-9A0A-091066D7ACC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15510" yWindow="2220" windowWidth="10785" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lineage Summary" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t>Variant</t>
   </si>
@@ -236,6 +236,12 @@
   </si>
   <si>
     <t>#254220</t>
+  </si>
+  <si>
+    <t>FL.1.5.1</t>
+  </si>
+  <si>
+    <t>#8cd17d</t>
   </si>
 </sst>
 </file>
@@ -1105,7 +1111,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -1400,6 +1406,14 @@
         <v>71</v>
       </c>
     </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1407,6 +1421,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="90bc503b-6eb4-4477-9236-230e894a8c79" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019EF3480BC5C5749AA11FB0475CF7A0F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9e8a1227a2a21758a504a4fbb7498eb4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd" xmlns:ns3="90bc503b-6eb4-4477-9236-230e894a8c79" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fa1332073f5f2190cdaadeed8648dd04" ns2:_="" ns3:_="">
     <xsd:import namespace="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd"/>
@@ -1623,17 +1648,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="90bc503b-6eb4-4477-9236-230e894a8c79" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1644,6 +1658,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D14E7338-C7ED-4988-977F-AB8C51D5B02E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd"/>
+    <ds:schemaRef ds:uri="90bc503b-6eb4-4477-9236-230e894a8c79"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26C3A01A-5B70-419B-9BF5-8E26874AB25B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1662,17 +1687,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D14E7338-C7ED-4988-977F-AB8C51D5B02E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd"/>
-    <ds:schemaRef ds:uri="90bc503b-6eb4-4477-9236-230e894a8c79"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECE872C0-CA59-4E8E-8928-E8AC0DA3AB58}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Production runs: 2023-08-15added GE.1, EG.6.1, XBB.1.16.11, FD.1.1 and XBB.1.5.70 as new lineage
</commit_message>
<xml_diff>
--- a/Lineage_Colors_on_CDT.xlsx
+++ b/Lineage_Colors_on_CDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\groups.biotech.cdc.gov\groups\Projects\SARS2Seq\repos\sc2_proportion_modeling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE603992-250F-4C6D-9A0A-091066D7ACC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0288ECCF-4D02-45B5-B55D-E84B01DB994A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t>Variant</t>
   </si>
@@ -242,6 +242,36 @@
   </si>
   <si>
     <t>#8cd17d</t>
+  </si>
+  <si>
+    <t>GE.1</t>
+  </si>
+  <si>
+    <t>#66534c</t>
+  </si>
+  <si>
+    <t>EG.6.1</t>
+  </si>
+  <si>
+    <t>#b9aba8</t>
+  </si>
+  <si>
+    <t>XBB.1.16.11</t>
+  </si>
+  <si>
+    <t>#d37295</t>
+  </si>
+  <si>
+    <t>FD.1.1</t>
+  </si>
+  <si>
+    <t>#e7cb40</t>
+  </si>
+  <si>
+    <t>XBB.1.5.70</t>
+  </si>
+  <si>
+    <t>#46783c</t>
   </si>
 </sst>
 </file>
@@ -1111,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -1414,6 +1444,46 @@
         <v>73</v>
       </c>
     </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" t="s">
+        <v>83</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1421,17 +1491,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="90bc503b-6eb4-4477-9236-230e894a8c79" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019EF3480BC5C5749AA11FB0475CF7A0F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9e8a1227a2a21758a504a4fbb7498eb4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd" xmlns:ns3="90bc503b-6eb4-4477-9236-230e894a8c79" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fa1332073f5f2190cdaadeed8648dd04" ns2:_="" ns3:_="">
     <xsd:import namespace="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd"/>
@@ -1648,6 +1707,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="90bc503b-6eb4-4477-9236-230e894a8c79" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1658,17 +1728,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D14E7338-C7ED-4988-977F-AB8C51D5B02E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd"/>
-    <ds:schemaRef ds:uri="90bc503b-6eb4-4477-9236-230e894a8c79"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26C3A01A-5B70-419B-9BF5-8E26874AB25B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1687,6 +1746,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D14E7338-C7ED-4988-977F-AB8C51D5B02E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="35115c8e-b0f9-4a59-ae7f-8ae068ab1fbd"/>
+    <ds:schemaRef ds:uri="90bc503b-6eb4-4477-9236-230e894a8c79"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECE872C0-CA59-4E8E-8928-E8AC0DA3AB58}">
   <ds:schemaRefs>

</xml_diff>